<commit_message>
Renomeia abas e artes ACA->ACAI (AÇAÍ) para bater com slug
</commit_message>
<xml_diff>
--- a/RELATÓRIO  - CAMPANHAS.xlsx
+++ b/RELATÓRIO  - CAMPANHAS.xlsx
@@ -5,19 +5,19 @@
   <sheets>
     <sheet name="10062026_VOUCHER_TV_45_89" sheetId="1" r:id="rId1"/>
     <sheet name="18062026_BATATAS_TV_45_120" sheetId="2" r:id="rId2"/>
-    <sheet name="22062026_ACA_TV_45_120" sheetId="3" r:id="rId3"/>
+    <sheet name="22062026_ACAI_TV_45_120" sheetId="3" r:id="rId3"/>
     <sheet name="23062026_BATATA_TV_45_120" sheetId="4" r:id="rId4"/>
     <sheet name="24062026_COPA_RP_20_44" sheetId="5" r:id="rId5"/>
-    <sheet name="25062026_DIADOACA_TV_45_120" sheetId="6" r:id="rId6"/>
-    <sheet name="26062026_DIADOACA_TV_45_120" sheetId="7" r:id="rId7"/>
+    <sheet name="25062026_DIADOACAI_TV_45_120" sheetId="6" r:id="rId6"/>
+    <sheet name="26062026_DIADOACAI_TV_45_120" sheetId="7" r:id="rId7"/>
     <sheet name="29062026_FECHAMENTO_TV_45_89" sheetId="8" r:id="rId8"/>
     <sheet name="30062026_PROSPECCAO_TV_45_365" sheetId="9" r:id="rId9"/>
     <sheet name="30062026_BRASILVENC_RP_20_44" sheetId="10" r:id="rId10"/>
     <sheet name="01072026_VOUCHER_TV_45_365" sheetId="11" r:id="rId11"/>
     <sheet name="02072026_VOLTEACOMP_RP_20_44" sheetId="12" r:id="rId12"/>
-    <sheet name="03072026_ACA_TV_45_120" sheetId="13" r:id="rId13"/>
-    <sheet name="06072026_ACA_TV_20_44" sheetId="14" r:id="rId14"/>
-    <sheet name="06072026_ACA_RP_20_44" sheetId="15" r:id="rId15"/>
+    <sheet name="03072026_ACAI_TV_45_120" sheetId="13" r:id="rId13"/>
+    <sheet name="06072026_ACAI_TV_20_44" sheetId="14" r:id="rId14"/>
+    <sheet name="06072026_ACAI_RP_20_44" sheetId="15" r:id="rId15"/>
     <sheet name="07072026_CNPJ_TV_44_365" sheetId="16" r:id="rId16"/>
     <sheet name="08072026_CNPJ_TV_45_400" sheetId="17" r:id="rId17"/>
     <sheet name="08072026_CNPJ_AT_20_44" sheetId="18" r:id="rId18"/>

</xml_diff>